<commit_message>
Fixed code after deletions, not finished
</commit_message>
<xml_diff>
--- a/tables/Parameters/AllParam.xlsx
+++ b/tables/Parameters/AllParam.xlsx
@@ -611,7 +611,7 @@
       </c>
       <c r="AL1" s="1" t="inlineStr">
         <is>
-          <t>Kx_error</t>
+          <t>Kx_err</t>
         </is>
       </c>
       <c r="AM1" s="1" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="AN1" s="1" t="inlineStr">
         <is>
-          <t>Kopt_error</t>
+          <t>Kopt_err</t>
         </is>
       </c>
       <c r="AO1" s="1" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="AP1" s="1" t="inlineStr">
         <is>
-          <t>q_error</t>
+          <t>q_err</t>
         </is>
       </c>
       <c r="AQ1" s="1" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="AR1" s="1" t="inlineStr">
         <is>
-          <t>Ohm_error</t>
+          <t>Ohm_err</t>
         </is>
       </c>
       <c r="AS1" s="1" t="inlineStr">
@@ -651,7 +651,7 @@
       </c>
       <c r="AT1" s="1" t="inlineStr">
         <is>
-          <t>i_error</t>
+          <t>i_err</t>
         </is>
       </c>
       <c r="AU1" s="1" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="AV1" s="1" t="inlineStr">
         <is>
-          <t>Mns_error</t>
+          <t>Mns_err</t>
         </is>
       </c>
       <c r="AW1" s="1" t="inlineStr">
@@ -671,7 +671,7 @@
       </c>
       <c r="AX1" s="1" t="inlineStr">
         <is>
-          <t>Mopt_error</t>
+          <t>Mopt_err</t>
         </is>
       </c>
       <c r="AY1" s="1" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="AZ1" s="1" t="inlineStr">
         <is>
-          <t>RL/a_error</t>
+          <t>RL/a_err</t>
         </is>
       </c>
       <c r="BA1" s="1" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="BB1" s="1" t="inlineStr">
         <is>
-          <t>a_error</t>
+          <t>a_err</t>
         </is>
       </c>
       <c r="BC1" s="1" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="BD1" s="1" t="inlineStr">
         <is>
-          <t>T0,ecl_error</t>
+          <t>T0,ecl_err</t>
         </is>
       </c>
       <c r="BE1" s="1" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="BF1" s="1" t="inlineStr">
         <is>
-          <t>Porb,ecl_error</t>
+          <t>Porb,ecl_err</t>
         </is>
       </c>
       <c r="BG1" s="1" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="BH1" s="1" t="inlineStr">
         <is>
-          <t>dtPorb_error</t>
+          <t>dtPorb_err</t>
         </is>
       </c>
       <c r="BI1" s="1" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="BJ1" s="1" t="inlineStr">
         <is>
-          <t>Orbital epoch_error</t>
+          <t>Orbital epoch_err</t>
         </is>
       </c>
       <c r="BK1" s="1" t="inlineStr">
@@ -746,7 +746,7 @@
       </c>
       <c r="BM1" s="1" t="inlineStr">
         <is>
-          <t>e_error</t>
+          <t>e_err</t>
         </is>
       </c>
       <c r="BN1" s="1" t="inlineStr">
@@ -756,7 +756,7 @@
       </c>
       <c r="BO1" s="1" t="inlineStr">
         <is>
-          <t>semi_eclipse_error</t>
+          <t>semi_eclipse_err</t>
         </is>
       </c>
       <c r="BP1" s="1" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="BQ1" s="1" t="inlineStr">
         <is>
-          <t>vsin(i)_error</t>
+          <t>vsin(i)_err</t>
         </is>
       </c>
       <c r="BR1" s="1" t="inlineStr">

</xml_diff>

<commit_message>
New BC for B stars
</commit_message>
<xml_diff>
--- a/tables/Parameters/AllParam.xlsx
+++ b/tables/Parameters/AllParam.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BT7"/>
+  <dimension ref="A1:BV7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,320 +466,330 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>V_err</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>BCv</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>(B-V)0</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Rv</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Rv_err</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Mbol</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Mv</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ST</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>L+</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>L-</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>d+</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>d-</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>Teff</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>Teff_err</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="Z1" s="1" t="inlineStr">
         <is>
           <t>Reff</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AA1" s="1" t="inlineStr">
         <is>
           <t>Reff+</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Reff-</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Ropt</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Ropt_err</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Rst</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Rst_err</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>RL</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>RL_err</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>RLq</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>RLq_err</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>RLg</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>RLg_err</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>Kx</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Kx_err</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Kopt</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Kopt_err</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>q</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>q_err</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Ohm</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Ohm_err</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>i</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>i_err</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>Mns</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>Mns_err</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Mopt</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>Mopt_err</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>RL/a</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>RL/a_err</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>a_err</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>T0,ecl</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>T0,ecl_err</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>Porb,ecl</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>Porb,ecl_err</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>dtPorb</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>dtPorb_err</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>Orbital epoch</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BL1" s="1" t="inlineStr">
         <is>
           <t>Orbital epoch_err</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>Ps</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BN1" s="1" t="inlineStr">
         <is>
           <t>e</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>e_err</t>
         </is>
       </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
         <is>
           <t>semi_eclipse</t>
         </is>
       </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BQ1" s="1" t="inlineStr">
         <is>
           <t>semi_eclipse_err</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>vsin(i)</t>
         </is>
       </c>
-      <c r="BQ1" s="1" t="inlineStr">
+      <c r="BS1" s="1" t="inlineStr">
         <is>
           <t>vsin(i)_err</t>
         </is>
       </c>
-      <c r="BR1" s="1" t="inlineStr">
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>Mhrd</t>
         </is>
       </c>
-      <c r="BS1" s="1" t="inlineStr">
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>Mhrd_err</t>
         </is>
       </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
         <is>
           <t>Lx</t>
         </is>
@@ -816,226 +826,232 @@
       <c r="H2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K2" t="inlineStr">
         <is>
           <t>-3.42</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>-0.27</t>
         </is>
       </c>
-      <c r="K2" t="n">
+      <c r="M2" t="n">
         <v>3.16</v>
       </c>
-      <c r="L2" t="n">
+      <c r="N2" t="n">
         <v>0.15</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>-8.50532122776198</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>-5.08532122776198</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>O6.5III</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>198668.261371504</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>44869.4476927578</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>33701.3277793123</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="U2" t="n">
         <v>6752.4946</v>
       </c>
-      <c r="T2" t="n">
+      <c r="V2" t="n">
         <v>678.6587</v>
       </c>
-      <c r="U2" t="n">
+      <c r="W2" t="n">
         <v>455.1382000000003</v>
       </c>
-      <c r="V2" t="n">
+      <c r="X2" t="n">
         <v>34500</v>
       </c>
-      <c r="W2" t="n">
+      <c r="Y2" t="n">
         <v>1000</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>12.4761106049604</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>1.58367109395482</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>1.28174948957142</t>
         </is>
       </c>
-      <c r="AA2" t="n">
+      <c r="AC2" t="n">
         <v>11.4</v>
       </c>
-      <c r="AB2" t="n">
+      <c r="AD2" t="n">
         <v>0.7</v>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>14.36</t>
         </is>
       </c>
-      <c r="AD2" t="n">
+      <c r="AF2" t="n">
         <v>2.154</v>
       </c>
-      <c r="AE2" t="n">
+      <c r="AG2" t="n">
         <v>12.726</v>
       </c>
-      <c r="AF2" t="n">
+      <c r="AH2" t="n">
         <v>0.3229674906240564</v>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>12.3332840935839</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>0.293733098903704</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>6.36984218288446</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>0.181277751759849</t>
         </is>
       </c>
-      <c r="AK2" t="n">
+      <c r="AM2" t="n">
         <v>414.317</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AN2" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="AM2" t="n">
+      <c r="AO2" t="n">
         <v>28</v>
       </c>
-      <c r="AN2" t="n">
+      <c r="AP2" t="n">
         <v>2</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="AQ2" t="n">
         <v>0.066</v>
       </c>
-      <c r="AP2" t="n">
+      <c r="AR2" t="n">
         <v>0.005</v>
       </c>
-      <c r="AQ2" t="n">
+      <c r="AS2" t="n">
         <v>0.75</v>
       </c>
-      <c r="AR2" t="n">
+      <c r="AT2" t="n">
         <v>0.13</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="AU2" t="n">
         <v>65</v>
       </c>
-      <c r="AT2" t="n">
+      <c r="AV2" t="n">
         <v>1</v>
       </c>
-      <c r="AU2" t="n">
+      <c r="AW2" t="n">
         <v>1.57</v>
       </c>
-      <c r="AV2" t="n">
+      <c r="AX2" t="n">
         <v>0.16</v>
       </c>
-      <c r="AW2" t="n">
+      <c r="AY2" t="n">
         <v>24</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="AZ2" t="n">
         <v>1</v>
       </c>
-      <c r="AY2" t="n">
+      <c r="BA2" t="n">
         <v>0.63</v>
       </c>
-      <c r="AZ2" t="n">
+      <c r="BB2" t="n">
         <v>0.01</v>
       </c>
-      <c r="BA2" t="n">
+      <c r="BC2" t="n">
         <v>20.2</v>
       </c>
-      <c r="BB2" t="n">
+      <c r="BD2" t="n">
         <v>0.4</v>
       </c>
-      <c r="BC2" t="n">
+      <c r="BE2" t="n">
         <v>50506.788423</v>
       </c>
-      <c r="BD2" t="n">
+      <c r="BF2" t="n">
         <v>7e-06</v>
       </c>
-      <c r="BE2" t="n">
+      <c r="BG2" t="n">
         <v>2.08704106</v>
       </c>
-      <c r="BF2" t="n">
+      <c r="BH2" t="n">
         <v>3e-08</v>
       </c>
-      <c r="BG2" t="n">
+      <c r="BI2" t="n">
         <v>-1.8</v>
       </c>
-      <c r="BH2" t="n">
+      <c r="BJ2" t="n">
         <v>0.001</v>
       </c>
-      <c r="BI2" t="n">
+      <c r="BK2" t="n">
         <v>50506.788423</v>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BL2" t="n">
         <v>7e-06</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BM2" t="n">
         <v>4.8</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BN2" t="n">
         <v>0.0016</v>
       </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="n">
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="n">
         <v>27.9</v>
       </c>
-      <c r="BO2" t="n">
+      <c r="BQ2" t="n">
         <v>0.3</v>
       </c>
-      <c r="BP2" t="n">
+      <c r="BR2" t="n">
         <v>204.8</v>
       </c>
-      <c r="BQ2" t="n">
+      <c r="BS2" t="n">
         <v>0.8</v>
       </c>
-      <c r="BR2" t="n">
+      <c r="BT2" t="n">
         <v>29</v>
       </c>
-      <c r="BS2" t="n">
+      <c r="BU2" t="n">
         <v>2</v>
       </c>
-      <c r="BT2" t="n">
+      <c r="BV2" t="n">
         <v>5e+37</v>
       </c>
     </row>
@@ -1070,228 +1086,232 @@
       <c r="H3" t="n">
         <v>0.02</v>
       </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>-2.7040000000000006</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
+      <c r="I3" t="n">
+        <v>14.35</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="K3" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="L3" t="inlineStr">
         <is>
           <t>-0.26</t>
         </is>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>3.16</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>0.15</v>
       </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>-9.20573104230982</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>-8.82173104230982</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>-6.50173104230982</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>B0.2Ia</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>378697.481532523</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>65928.0469495372</t>
-        </is>
-      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>75599.1428067363</t>
-        </is>
-      </c>
-      <c r="S3" t="n">
+          <t>265884.130512809</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>46288.1912196714</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>53078.2836773541</t>
+        </is>
+      </c>
+      <c r="U3" t="n">
         <v>5535.3643</v>
       </c>
-      <c r="T3" t="n">
+      <c r="V3" t="n">
         <v>352.5882999999994</v>
       </c>
-      <c r="U3" t="n">
+      <c r="W3" t="n">
         <v>444.3267000000005</v>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>24000</v>
       </c>
-      <c r="W3" t="n">
+      <c r="Y3" t="n">
         <v>1000</v>
       </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>35.5940073597207</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>4.28924993559849</t>
-        </is>
-      </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>4.62823618030184</t>
-        </is>
-      </c>
-      <c r="AA3" t="n">
+          <t>29.8247550772236</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>3.59402714904720</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>3.87806883113850</t>
+        </is>
+      </c>
+      <c r="AC3" t="n">
         <v>13</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AD3" t="n">
         <v>1</v>
       </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AE3" t="inlineStr">
         <is>
           <t>22.599999999999994</t>
         </is>
       </c>
-      <c r="AD3" t="n">
+      <c r="AF3" t="n">
         <v>3.389999999999999</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AG3" t="n">
         <v>11.66</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AH3" t="n">
         <v>0.8464632301523793</v>
       </c>
-      <c r="AG3" t="inlineStr">
+      <c r="AI3" t="inlineStr">
         <is>
           <t>13.4738464692258</t>
         </is>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>0.697890522579867</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AK3" t="inlineStr">
         <is>
           <t>7.96322282646401</t>
         </is>
       </c>
-      <c r="AJ3" t="inlineStr">
+      <c r="AL3" t="inlineStr">
         <is>
           <t>0.457908402696324</t>
         </is>
       </c>
-      <c r="AK3" t="n">
+      <c r="AM3" t="n">
         <v>316</v>
       </c>
-      <c r="AL3" t="n">
+      <c r="AN3" t="n">
         <v>10</v>
       </c>
-      <c r="AM3" t="n">
+      <c r="AO3" t="n">
         <v>20</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="AP3" t="n">
         <v>3</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="AQ3" t="n">
         <v>0.06</v>
       </c>
-      <c r="AP3" t="n">
+      <c r="AR3" t="n">
         <v>0.01</v>
       </c>
-      <c r="AQ3" t="n">
+      <c r="AS3" t="n">
         <v>0.91</v>
       </c>
-      <c r="AR3" t="n">
+      <c r="AT3" t="n">
         <v>0.2</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="AU3" t="n">
         <v>67</v>
       </c>
-      <c r="AT3" t="n">
+      <c r="AV3" t="n">
         <v>1</v>
       </c>
-      <c r="AU3" t="n">
+      <c r="AW3" t="n">
         <v>1.02</v>
       </c>
-      <c r="AV3" t="n">
+      <c r="AX3" t="n">
         <v>0.17</v>
       </c>
-      <c r="AW3" t="n">
+      <c r="AY3" t="n">
         <v>16</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="AZ3" t="n">
         <v>2</v>
       </c>
-      <c r="AY3" t="n">
+      <c r="BA3" t="n">
         <v>0.53</v>
       </c>
-      <c r="AZ3" t="n">
+      <c r="BB3" t="n">
         <v>0.03</v>
       </c>
-      <c r="BA3" t="n">
+      <c r="BC3" t="n">
         <v>22</v>
       </c>
-      <c r="BB3" t="n">
+      <c r="BD3" t="n">
         <v>1</v>
       </c>
-      <c r="BC3" t="n">
+      <c r="BE3" t="n">
         <v>52855.061</v>
       </c>
-      <c r="BD3" t="n">
+      <c r="BF3" t="n">
         <v>0.013</v>
       </c>
-      <c r="BE3" t="n">
+      <c r="BG3" t="n">
         <v>3.728414</v>
       </c>
-      <c r="BF3" t="n">
+      <c r="BH3" t="n">
         <v>7.6e-06</v>
       </c>
-      <c r="BG3" t="n">
+      <c r="BI3" t="n">
         <v>-0.7</v>
       </c>
-      <c r="BH3" t="n">
+      <c r="BJ3" t="n">
         <v>0.8</v>
       </c>
-      <c r="BI3" t="n">
+      <c r="BK3" t="n">
         <v>52851.33</v>
       </c>
-      <c r="BJ3" t="n">
+      <c r="BL3" t="n">
         <v>0.01</v>
       </c>
-      <c r="BK3" t="n">
+      <c r="BM3" t="n">
         <v>526.8</v>
       </c>
-      <c r="BL3" t="n">
+      <c r="BN3" t="n">
         <v>0.18</v>
       </c>
-      <c r="BM3" t="n">
+      <c r="BO3" t="n">
         <v>0.01</v>
       </c>
-      <c r="BN3" t="n">
+      <c r="BP3" t="n">
         <v>21</v>
       </c>
-      <c r="BO3" t="n">
+      <c r="BQ3" t="n">
         <v>1</v>
       </c>
-      <c r="BP3" t="n">
+      <c r="BR3" t="n">
         <v>224.9</v>
       </c>
-      <c r="BQ3" t="n">
+      <c r="BS3" t="n">
         <v>0.7</v>
       </c>
-      <c r="BR3" t="n">
+      <c r="BT3" t="n">
         <v>35</v>
       </c>
-      <c r="BS3" t="n">
+      <c r="BU3" t="n">
         <v>2</v>
       </c>
-      <c r="BT3" t="n">
+      <c r="BV3" t="n">
         <v>2e+36</v>
       </c>
     </row>
@@ -1326,218 +1346,224 @@
       <c r="H4" t="n">
         <v>0</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I4" t="n">
+        <v>6.54</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>-3.32</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>-0.27</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>3.16</v>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>0.15</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>-9.34461962281793</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>-6.02461962281793</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>O6.5Iaf+</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>430375.806074179</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>59772.8357455441</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>49829.8400709757</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="U4" t="n">
         <v>1513.9932</v>
       </c>
-      <c r="T4" t="n">
+      <c r="V4" t="n">
         <v>78.38200000000006</v>
       </c>
-      <c r="U4" t="n">
+      <c r="W4" t="n">
         <v>52.65149999999994</v>
       </c>
-      <c r="V4" t="n">
+      <c r="X4" t="n">
         <v>35895</v>
       </c>
-      <c r="W4" t="n">
+      <c r="Y4" t="n">
         <v>1000</v>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>16.9632541964421</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>1.51028021716036</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>1.36297188049476</t>
         </is>
       </c>
-      <c r="AA4" t="n">
+      <c r="AC4" t="n">
         <v>22</v>
       </c>
-      <c r="AB4" t="n">
+      <c r="AD4" t="n">
         <v>2</v>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>20.22</t>
         </is>
       </c>
-      <c r="AD4" t="n">
+      <c r="AF4" t="n">
         <v>3.033</v>
       </c>
-      <c r="AE4" t="n">
+      <c r="AG4" t="n">
         <v>24.29</v>
       </c>
-      <c r="AF4" t="n">
+      <c r="AH4" t="n">
         <v>0.7250765476830705</v>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>22.4221610513527</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>0.725547330706974</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>11.0576539439844</t>
         </is>
       </c>
-      <c r="AJ4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>0.534214506648961</t>
         </is>
       </c>
-      <c r="AK4" t="n">
+      <c r="AM4" t="n">
         <v>435</v>
       </c>
-      <c r="AL4" t="n">
+      <c r="AN4" t="n">
         <v>10</v>
       </c>
-      <c r="AM4" t="n">
+      <c r="AO4" t="n">
         <v>19</v>
       </c>
-      <c r="AN4" t="n">
+      <c r="AP4" t="n">
         <v>1</v>
       </c>
-      <c r="AO4" t="n">
+      <c r="AQ4" t="n">
         <v>0.043</v>
       </c>
-      <c r="AP4" t="n">
+      <c r="AR4" t="n">
         <v>0.002</v>
       </c>
-      <c r="AQ4" t="n">
+      <c r="AS4" t="n">
         <v>0.47</v>
       </c>
-      <c r="AR4" t="n">
+      <c r="AT4" t="n">
         <v>0.04</v>
       </c>
-      <c r="AS4" t="n">
+      <c r="AU4" t="n">
         <v>62</v>
       </c>
-      <c r="AT4" t="n">
+      <c r="AV4" t="n">
         <v>1</v>
       </c>
-      <c r="AU4" t="n">
+      <c r="AW4" t="n">
         <v>1.96</v>
       </c>
-      <c r="AV4" t="n">
+      <c r="AX4" t="n">
         <v>0.19</v>
       </c>
-      <c r="AW4" t="n">
+      <c r="AY4" t="n">
         <v>46</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="AZ4" t="n">
         <v>5</v>
       </c>
-      <c r="AY4" t="n">
+      <c r="BA4" t="n">
         <v>0.694</v>
       </c>
-      <c r="AZ4" t="n">
+      <c r="BB4" t="n">
         <v>0.006</v>
       </c>
-      <c r="BA4" t="n">
+      <c r="BC4" t="n">
         <v>35</v>
       </c>
-      <c r="BB4" t="n">
+      <c r="BD4" t="n">
         <v>1</v>
       </c>
-      <c r="BC4" t="n">
+      <c r="BE4" t="n">
         <v>53785.85</v>
       </c>
-      <c r="BD4" t="n">
+      <c r="BF4" t="n">
         <v>0.007</v>
       </c>
-      <c r="BE4" t="n">
+      <c r="BG4" t="n">
         <v>3.411581</v>
       </c>
-      <c r="BF4" t="n">
+      <c r="BH4" t="n">
         <v>7e-06</v>
       </c>
-      <c r="BG4" t="n">
+      <c r="BI4" t="n">
         <v>-1.6</v>
       </c>
-      <c r="BH4" t="n">
+      <c r="BJ4" t="n">
         <v>0.1</v>
       </c>
-      <c r="BI4" t="n">
+      <c r="BK4" t="n">
         <v>48900.373</v>
       </c>
-      <c r="BJ4" t="n">
+      <c r="BL4" t="n">
         <v>0.015</v>
       </c>
-      <c r="BK4" t="inlineStr"/>
-      <c r="BL4" t="inlineStr"/>
       <c r="BM4" t="inlineStr"/>
-      <c r="BN4" t="n">
+      <c r="BN4" t="inlineStr"/>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="n">
         <v>32</v>
       </c>
-      <c r="BO4" t="n">
+      <c r="BQ4" t="n">
         <v>1</v>
       </c>
-      <c r="BP4" t="inlineStr"/>
-      <c r="BQ4" t="inlineStr"/>
-      <c r="BR4" t="n">
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="n">
         <v>44</v>
       </c>
-      <c r="BS4" t="n">
+      <c r="BU4" t="n">
         <v>2</v>
       </c>
-      <c r="BT4" t="n">
+      <c r="BV4" t="n">
         <v>9.800000000000001e+35</v>
       </c>
     </row>
@@ -1572,228 +1598,234 @@
       <c r="H5" t="n">
         <v>0.01</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I5" t="n">
+        <v>14</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>-3.16</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>-0.27</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>3.4</v>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>0</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>-7.72873449531503</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>-4.56873449531503</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>O8III</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>97161.4076496157</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>18580.6987382659</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>18580.6987382659</t>
         </is>
       </c>
-      <c r="S5" t="n">
+      <c r="U5" t="n">
         <v>48590</v>
       </c>
-      <c r="T5" t="n">
+      <c r="V5" t="n">
         <v>4000</v>
       </c>
-      <c r="U5" t="n">
+      <c r="W5" t="n">
         <v>4000</v>
       </c>
-      <c r="V5" t="n">
+      <c r="X5" t="n">
         <v>32573</v>
       </c>
-      <c r="W5" t="n">
+      <c r="Y5" t="n">
         <v>1000</v>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>9.78778771242834</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>1.11222907861592</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>1.11222907861592</t>
         </is>
       </c>
-      <c r="AA5" t="n">
+      <c r="AC5" t="n">
         <v>7.4</v>
       </c>
-      <c r="AB5" t="n">
+      <c r="AD5" t="n">
         <v>0.4</v>
       </c>
-      <c r="AC5" t="inlineStr">
+      <c r="AE5" t="inlineStr">
         <is>
           <t>13.74</t>
         </is>
       </c>
-      <c r="AD5" t="n">
+      <c r="AF5" t="n">
         <v>2.061</v>
       </c>
-      <c r="AE5" t="n">
+      <c r="AG5" t="n">
         <v>8.377999999999998</v>
       </c>
-      <c r="AF5" t="n">
+      <c r="AH5" t="n">
         <v>0.1846293584455083</v>
       </c>
-      <c r="AG5" t="inlineStr">
+      <c r="AI5" t="inlineStr">
         <is>
           <t>8.36188984223463</t>
         </is>
       </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AJ5" t="inlineStr">
         <is>
           <t>0.153362041572946</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
+      <c r="AK5" t="inlineStr">
         <is>
           <t>4.29964416954258</t>
         </is>
       </c>
-      <c r="AJ5" t="inlineStr">
+      <c r="AL5" t="inlineStr">
         <is>
           <t>0.113170143887694</t>
         </is>
       </c>
-      <c r="AK5" t="n">
+      <c r="AM5" t="n">
         <v>407.8</v>
       </c>
-      <c r="AL5" t="n">
+      <c r="AN5" t="n">
         <v>0.3</v>
       </c>
-      <c r="AM5" t="n">
+      <c r="AO5" t="n">
         <v>35</v>
       </c>
-      <c r="AN5" t="n">
+      <c r="AP5" t="n">
         <v>2</v>
       </c>
-      <c r="AO5" t="n">
+      <c r="AQ5" t="n">
         <v>0.08599999999999999</v>
       </c>
-      <c r="AP5" t="n">
+      <c r="AR5" t="n">
         <v>0.004</v>
       </c>
-      <c r="AQ5" t="n">
+      <c r="AS5" t="n">
         <v>0.97</v>
       </c>
-      <c r="AR5" t="n">
+      <c r="AT5" t="n">
         <v>0.13</v>
       </c>
-      <c r="AS5" t="n">
+      <c r="AU5" t="n">
         <v>59.3</v>
       </c>
-      <c r="AT5" t="n">
+      <c r="AV5" t="n">
         <v>0.9</v>
       </c>
-      <c r="AU5" t="n">
+      <c r="AW5" t="n">
         <v>1.57</v>
       </c>
-      <c r="AV5" t="n">
+      <c r="AX5" t="n">
         <v>0.11</v>
       </c>
-      <c r="AW5" t="n">
+      <c r="AY5" t="n">
         <v>18</v>
       </c>
-      <c r="AX5" t="n">
+      <c r="AZ5" t="n">
         <v>1</v>
       </c>
-      <c r="AY5" t="n">
+      <c r="BA5" t="n">
         <v>0.59</v>
       </c>
-      <c r="AZ5" t="n">
+      <c r="BB5" t="n">
         <v>0.01</v>
       </c>
-      <c r="BA5" t="n">
+      <c r="BC5" t="n">
         <v>14.2</v>
       </c>
-      <c r="BB5" t="n">
+      <c r="BD5" t="n">
         <v>0.2</v>
       </c>
-      <c r="BC5" t="n">
+      <c r="BE5" t="n">
         <v>53013.591</v>
       </c>
-      <c r="BD5" t="n">
+      <c r="BF5" t="n">
         <v>0.0008</v>
       </c>
-      <c r="BE5" t="n">
+      <c r="BG5" t="n">
         <v>1.408379</v>
       </c>
-      <c r="BF5" t="n">
+      <c r="BH5" t="n">
         <v>7e-07</v>
       </c>
-      <c r="BG5" t="n">
+      <c r="BI5" t="n">
         <v>-1</v>
       </c>
-      <c r="BH5" t="n">
+      <c r="BJ5" t="n">
         <v>0.05</v>
       </c>
-      <c r="BI5" t="n">
+      <c r="BK5" t="n">
         <v>51110.86579</v>
       </c>
-      <c r="BJ5" t="n">
+      <c r="BL5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="BK5" t="n">
+      <c r="BM5" t="n">
         <v>13.5</v>
       </c>
-      <c r="BL5" t="n">
+      <c r="BN5" t="n">
         <v>0.006</v>
       </c>
-      <c r="BM5" t="n">
+      <c r="BO5" t="n">
         <v>0.002</v>
       </c>
-      <c r="BN5" t="n">
+      <c r="BP5" t="n">
         <v>15.8</v>
       </c>
-      <c r="BO5" t="n">
+      <c r="BQ5" t="n">
         <v>0.8</v>
       </c>
-      <c r="BP5" t="n">
+      <c r="BR5" t="n">
         <v>257.9</v>
       </c>
-      <c r="BQ5" t="n">
+      <c r="BS5" t="n">
         <v>0.7</v>
       </c>
-      <c r="BR5" t="n">
+      <c r="BT5" t="n">
         <v>22</v>
       </c>
-      <c r="BS5" t="n">
+      <c r="BU5" t="n">
         <v>1</v>
       </c>
-      <c r="BT5" t="n">
+      <c r="BV5" t="n">
         <v>2.2e+38</v>
       </c>
     </row>
@@ -1828,228 +1860,232 @@
       <c r="H6" t="n">
         <v>0.01</v>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>-2.74</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
+      <c r="I6" t="n">
+        <v>13.15</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-2.35</v>
+      </c>
+      <c r="L6" t="inlineStr">
         <is>
           <t>-0.26</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="M6" t="n">
         <v>2.53</v>
       </c>
-      <c r="L6" t="n">
+      <c r="N6" t="n">
         <v>0</v>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>-8.84561447195190</t>
-        </is>
-      </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>-8.45561447195190</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
         <is>
           <t>-6.10561447195190</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>B0Ib</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>271797.707162782</t>
-        </is>
-      </c>
-      <c r="Q6" t="inlineStr">
-        <is>
-          <t>43425.0412462522</t>
-        </is>
-      </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>43425.0412462522</t>
-        </is>
-      </c>
-      <c r="S6" t="n">
+          <t>189777.966494933</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>30320.7709465210</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>30320.7709465210</t>
+        </is>
+      </c>
+      <c r="U6" t="n">
         <v>62440</v>
       </c>
-      <c r="T6" t="n">
+      <c r="V6" t="n">
         <v>4000</v>
       </c>
-      <c r="U6" t="n">
+      <c r="W6" t="n">
         <v>4000</v>
       </c>
-      <c r="V6" t="n">
+      <c r="X6" t="n">
         <v>24380</v>
       </c>
-      <c r="W6" t="n">
+      <c r="Y6" t="n">
         <v>1000</v>
       </c>
-      <c r="X6" t="inlineStr">
-        <is>
-          <t>29.2219136230177</t>
-        </is>
-      </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>3.34603567974393</t>
-        </is>
-      </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>3.34603567974393</t>
-        </is>
-      </c>
-      <c r="AA6" t="n">
+          <t>24.4179192218864</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>2.79595751310347</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>2.79595751310347</t>
+        </is>
+      </c>
+      <c r="AC6" t="n">
         <v>15</v>
       </c>
-      <c r="AB6" t="n">
+      <c r="AD6" t="n">
         <v>1</v>
       </c>
-      <c r="AC6" t="inlineStr">
+      <c r="AE6" t="inlineStr">
         <is>
           <t>22.459999999999997</t>
         </is>
       </c>
-      <c r="AD6" t="n">
+      <c r="AF6" t="n">
         <v>3.368999999999999</v>
       </c>
-      <c r="AE6" t="n">
+      <c r="AG6" t="n">
         <v>17.019</v>
       </c>
-      <c r="AF6" t="n">
+      <c r="AH6" t="n">
         <v>0.7026329055773007</v>
       </c>
-      <c r="AG6" t="inlineStr">
+      <c r="AI6" t="inlineStr">
         <is>
           <t>16.9786936673335</t>
         </is>
       </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>0.524823344586292</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr">
+      <c r="AK6" t="inlineStr">
         <is>
           <t>10.1601686470543</t>
         </is>
       </c>
-      <c r="AJ6" t="inlineStr">
+      <c r="AL6" t="inlineStr">
         <is>
           <t>0.404455984912469</t>
         </is>
       </c>
-      <c r="AK6" t="n">
+      <c r="AM6" t="n">
         <v>299.631</v>
       </c>
-      <c r="AL6" t="n">
+      <c r="AN6" t="n">
         <v>0.005</v>
       </c>
-      <c r="AM6" t="n">
+      <c r="AO6" t="n">
         <v>20</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="AP6" t="n">
         <v>1</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="AQ6" t="n">
         <v>0.067</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="AR6" t="n">
         <v>0.004</v>
       </c>
-      <c r="AQ6" t="n">
+      <c r="AS6" t="n">
         <v>0.91</v>
       </c>
-      <c r="AR6" t="n">
+      <c r="AT6" t="n">
         <v>0.2</v>
       </c>
-      <c r="AS6" t="n">
+      <c r="AU6" t="n">
         <v>62</v>
       </c>
-      <c r="AT6" t="n">
+      <c r="AV6" t="n">
         <v>2</v>
       </c>
-      <c r="AU6" t="n">
+      <c r="AW6" t="n">
         <v>1.21</v>
       </c>
-      <c r="AV6" t="n">
+      <c r="AX6" t="n">
         <v>0.12</v>
       </c>
-      <c r="AW6" t="n">
+      <c r="AY6" t="n">
         <v>18</v>
       </c>
-      <c r="AX6" t="n">
+      <c r="AZ6" t="n">
         <v>2</v>
       </c>
-      <c r="AY6" t="n">
+      <c r="BA6" t="n">
         <v>0.61</v>
       </c>
-      <c r="AZ6" t="n">
+      <c r="BB6" t="n">
         <v>0.02</v>
       </c>
-      <c r="BA6" t="n">
+      <c r="BC6" t="n">
         <v>27.9</v>
       </c>
-      <c r="BB6" t="n">
+      <c r="BD6" t="n">
         <v>0.7</v>
       </c>
-      <c r="BC6" t="n">
+      <c r="BE6" t="n">
         <v>52846.68881</v>
       </c>
-      <c r="BD6" t="n">
+      <c r="BF6" t="n">
         <v>2.4e-05</v>
       </c>
-      <c r="BE6" t="n">
+      <c r="BG6" t="n">
         <v>3.89192316</v>
       </c>
-      <c r="BF6" t="n">
+      <c r="BH6" t="n">
         <v>6.6e-08</v>
       </c>
-      <c r="BG6" t="n">
+      <c r="BI6" t="n">
         <v>-3.541</v>
       </c>
-      <c r="BH6" t="n">
+      <c r="BJ6" t="n">
         <v>0.002</v>
       </c>
-      <c r="BI6" t="n">
+      <c r="BK6" t="n">
         <v>50324.691861</v>
       </c>
-      <c r="BJ6" t="n">
+      <c r="BL6" t="n">
         <v>8e-06</v>
       </c>
-      <c r="BK6" t="n">
+      <c r="BM6" t="n">
         <v>0.71</v>
       </c>
-      <c r="BL6" t="n">
+      <c r="BN6" t="n">
         <v>0.0008899999999999999</v>
       </c>
-      <c r="BM6" t="n">
+      <c r="BO6" t="n">
         <v>6e-05</v>
       </c>
-      <c r="BN6" t="n">
+      <c r="BP6" t="n">
         <v>23</v>
       </c>
-      <c r="BO6" t="n">
+      <c r="BQ6" t="n">
         <v>2</v>
       </c>
-      <c r="BP6" t="n">
+      <c r="BR6" t="n">
         <v>178</v>
       </c>
-      <c r="BQ6" t="n">
+      <c r="BS6" t="n">
         <v>0.8</v>
       </c>
-      <c r="BR6" t="n">
+      <c r="BT6" t="n">
         <v>29</v>
       </c>
-      <c r="BS6" t="n">
+      <c r="BU6" t="n">
         <v>2</v>
       </c>
-      <c r="BT6" t="n">
+      <c r="BV6" t="n">
         <v>2.6e+38</v>
       </c>
     </row>
@@ -2084,228 +2120,232 @@
       <c r="H7" t="n">
         <v>0</v>
       </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>-2.6500000000000004</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
+      <c r="I7" t="n">
+        <v>6.87</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-2.16</v>
+      </c>
+      <c r="L7" t="inlineStr">
         <is>
           <t>-0.26</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="M7" t="n">
         <v>3.16</v>
       </c>
-      <c r="L7" t="n">
+      <c r="N7" t="n">
         <v>0.15</v>
       </c>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>-9.68375611051318</t>
-        </is>
-      </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>-9.19375611051318</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
         <is>
           <t>-7.03375611051318</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>B0.5Iae</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>588169.424345731</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>64991.2299955974</t>
-        </is>
-      </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>67721.9679443754</t>
-        </is>
-      </c>
-      <c r="S7" t="n">
+          <t>374543.654958348</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>41386.1241594926</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>43125.0458540477</t>
+        </is>
+      </c>
+      <c r="U7" t="n">
         <v>1969.4784</v>
       </c>
-      <c r="T7" t="n">
+      <c r="V7" t="n">
         <v>60.11470000000008</v>
       </c>
-      <c r="U7" t="n">
+      <c r="W7" t="n">
         <v>68.04140000000007</v>
       </c>
-      <c r="V7" t="n">
+      <c r="X7" t="n">
         <v>22370</v>
       </c>
-      <c r="W7" t="n">
+      <c r="Y7" t="n">
         <v>1000</v>
       </c>
-      <c r="X7" t="inlineStr">
-        <is>
-          <t>51.0590129277988</t>
-        </is>
-      </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>5.36624093989413</t>
-        </is>
-      </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>5.42948536137474</t>
-        </is>
-      </c>
-      <c r="AA7" t="n">
+          <t>40.7448210535303</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>4.28223176063543</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>4.33270047297629</t>
+        </is>
+      </c>
+      <c r="AC7" t="n">
         <v>29</v>
       </c>
-      <c r="AB7" t="n">
+      <c r="AD7" t="n">
         <v>1</v>
       </c>
-      <c r="AC7" t="inlineStr">
+      <c r="AE7" t="inlineStr">
         <is>
           <t>22.809999999999995</t>
         </is>
       </c>
-      <c r="AD7" t="n">
+      <c r="AF7" t="n">
         <v>3.421499999999999</v>
       </c>
-      <c r="AE7" t="n">
+      <c r="AG7" t="n">
         <v>35.462</v>
       </c>
-      <c r="AF7" t="n">
+      <c r="AH7" t="n">
         <v>0.5489535590557729</v>
       </c>
-      <c r="AG7" t="inlineStr">
+      <c r="AI7" t="inlineStr">
         <is>
           <t>35.4052971460730</t>
         </is>
       </c>
-      <c r="AH7" t="inlineStr">
+      <c r="AJ7" t="inlineStr">
         <is>
           <t>0.567412643709415</t>
         </is>
       </c>
-      <c r="AI7" t="inlineStr">
+      <c r="AK7" t="inlineStr">
         <is>
           <t>23.2133018271434</t>
         </is>
       </c>
-      <c r="AJ7" t="inlineStr">
+      <c r="AL7" t="inlineStr">
         <is>
           <t>0.381892414835567</t>
         </is>
       </c>
-      <c r="AK7" t="n">
+      <c r="AM7" t="n">
         <v>278.1</v>
       </c>
-      <c r="AL7" t="n">
+      <c r="AN7" t="n">
         <v>0.3</v>
       </c>
-      <c r="AM7" t="n">
+      <c r="AO7" t="n">
         <v>23</v>
       </c>
-      <c r="AN7" t="n">
+      <c r="AP7" t="n">
         <v>2</v>
       </c>
-      <c r="AO7" t="n">
+      <c r="AQ7" t="n">
         <v>0.081</v>
       </c>
-      <c r="AP7" t="n">
+      <c r="AR7" t="n">
         <v>0.005</v>
       </c>
-      <c r="AQ7" t="n">
+      <c r="AS7" t="n">
         <v>0.67</v>
       </c>
-      <c r="AR7" t="n">
+      <c r="AT7" t="n">
         <v>0.04</v>
       </c>
-      <c r="AS7" t="n">
+      <c r="AU7" t="n">
         <v>72.8</v>
       </c>
-      <c r="AT7" t="n">
+      <c r="AV7" t="n">
         <v>0.4</v>
       </c>
-      <c r="AU7" t="n">
+      <c r="AW7" t="n">
         <v>2.12</v>
       </c>
-      <c r="AV7" t="n">
+      <c r="AX7" t="n">
         <v>0.16</v>
       </c>
-      <c r="AW7" t="n">
+      <c r="AY7" t="n">
         <v>26</v>
       </c>
-      <c r="AX7" t="n">
+      <c r="AZ7" t="n">
         <v>1</v>
       </c>
-      <c r="AY7" t="n">
+      <c r="BA7" t="n">
         <v>0.595</v>
       </c>
-      <c r="AZ7" t="n">
+      <c r="BB7" t="n">
         <v>0.006</v>
       </c>
-      <c r="BA7" t="n">
+      <c r="BC7" t="n">
         <v>59.6</v>
       </c>
-      <c r="BB7" t="n">
+      <c r="BD7" t="n">
         <v>0.7</v>
       </c>
-      <c r="BC7" t="n">
+      <c r="BE7" t="n">
         <v>42611.349</v>
       </c>
-      <c r="BD7" t="n">
+      <c r="BF7" t="n">
         <v>0.013</v>
       </c>
-      <c r="BE7" t="n">
+      <c r="BG7" t="n">
         <v>8.964427000000001</v>
       </c>
-      <c r="BF7" t="n">
+      <c r="BH7" t="n">
         <v>1.2e-05</v>
       </c>
-      <c r="BG7" t="n">
+      <c r="BI7" t="n">
         <v>-0.1</v>
       </c>
-      <c r="BH7" t="n">
+      <c r="BJ7" t="n">
         <v>0.3</v>
       </c>
-      <c r="BI7" t="n">
+      <c r="BK7" t="n">
         <v>48895.2186</v>
       </c>
-      <c r="BJ7" t="n">
+      <c r="BL7" t="n">
         <v>0.0012</v>
       </c>
-      <c r="BK7" t="n">
+      <c r="BM7" t="n">
         <v>283.2</v>
       </c>
-      <c r="BL7" t="n">
+      <c r="BN7" t="n">
         <v>0.0898</v>
       </c>
-      <c r="BM7" t="n">
+      <c r="BO7" t="n">
         <v>0.0012</v>
       </c>
-      <c r="BN7" t="n">
+      <c r="BP7" t="n">
         <v>30.5</v>
       </c>
-      <c r="BO7" t="n">
+      <c r="BQ7" t="n">
         <v>0.1</v>
       </c>
-      <c r="BP7" t="n">
+      <c r="BR7" t="n">
         <v>130.3</v>
       </c>
-      <c r="BQ7" t="n">
+      <c r="BS7" t="n">
         <v>0.2</v>
       </c>
-      <c r="BR7" t="n">
+      <c r="BT7" t="n">
         <v>42</v>
       </c>
-      <c r="BS7" t="n">
+      <c r="BU7" t="n">
         <v>2</v>
       </c>
-      <c r="BT7" t="n">
+      <c r="BV7" t="n">
         <v>4.6e+36</v>
       </c>
     </row>

</xml_diff>

<commit_message>
New spectra for Vela X-1 and 4U1700-37. Selected new lines for the model fit. TODO: Run model fit.
</commit_message>
<xml_diff>
--- a/tables/Parameters/AllParam.xlsx
+++ b/tables/Parameters/AllParam.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BV7"/>
+  <dimension ref="A1:BW7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -551,245 +551,250 @@
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
+          <t>Teff_model</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>Reff</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Reff+</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Reff-</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AD1" s="1" t="inlineStr">
         <is>
           <t>Ropt</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AE1" s="1" t="inlineStr">
         <is>
           <t>Ropt_err</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AF1" s="1" t="inlineStr">
         <is>
           <t>Rst</t>
         </is>
       </c>
-      <c r="AF1" s="1" t="inlineStr">
+      <c r="AG1" s="1" t="inlineStr">
         <is>
           <t>Rst_err</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t>RL</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>RL_err</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>RLq</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>RLq_err</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>RLg</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>RLg_err</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>Kx</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>Kx_err</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>Kopt</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>Kopt_err</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>q</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>q_err</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Ohm</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Ohm_err</t>
         </is>
       </c>
-      <c r="AU1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>i</t>
         </is>
       </c>
-      <c r="AV1" s="1" t="inlineStr">
+      <c r="AW1" s="1" t="inlineStr">
         <is>
           <t>i_err</t>
         </is>
       </c>
-      <c r="AW1" s="1" t="inlineStr">
+      <c r="AX1" s="1" t="inlineStr">
         <is>
           <t>Mns</t>
         </is>
       </c>
-      <c r="AX1" s="1" t="inlineStr">
+      <c r="AY1" s="1" t="inlineStr">
         <is>
           <t>Mns_err</t>
         </is>
       </c>
-      <c r="AY1" s="1" t="inlineStr">
+      <c r="AZ1" s="1" t="inlineStr">
         <is>
           <t>Mopt</t>
         </is>
       </c>
-      <c r="AZ1" s="1" t="inlineStr">
+      <c r="BA1" s="1" t="inlineStr">
         <is>
           <t>Mopt_err</t>
         </is>
       </c>
-      <c r="BA1" s="1" t="inlineStr">
+      <c r="BB1" s="1" t="inlineStr">
         <is>
           <t>RL/a</t>
         </is>
       </c>
-      <c r="BB1" s="1" t="inlineStr">
+      <c r="BC1" s="1" t="inlineStr">
         <is>
           <t>RL/a_err</t>
         </is>
       </c>
-      <c r="BC1" s="1" t="inlineStr">
+      <c r="BD1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="BD1" s="1" t="inlineStr">
+      <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>a_err</t>
         </is>
       </c>
-      <c r="BE1" s="1" t="inlineStr">
+      <c r="BF1" s="1" t="inlineStr">
         <is>
           <t>T0,ecl</t>
         </is>
       </c>
-      <c r="BF1" s="1" t="inlineStr">
+      <c r="BG1" s="1" t="inlineStr">
         <is>
           <t>T0,ecl_err</t>
         </is>
       </c>
-      <c r="BG1" s="1" t="inlineStr">
+      <c r="BH1" s="1" t="inlineStr">
         <is>
           <t>Porb,ecl</t>
         </is>
       </c>
-      <c r="BH1" s="1" t="inlineStr">
+      <c r="BI1" s="1" t="inlineStr">
         <is>
           <t>Porb,ecl_err</t>
         </is>
       </c>
-      <c r="BI1" s="1" t="inlineStr">
+      <c r="BJ1" s="1" t="inlineStr">
         <is>
           <t>dtPorb</t>
         </is>
       </c>
-      <c r="BJ1" s="1" t="inlineStr">
+      <c r="BK1" s="1" t="inlineStr">
         <is>
           <t>dtPorb_err</t>
         </is>
       </c>
-      <c r="BK1" s="1" t="inlineStr">
+      <c r="BL1" s="1" t="inlineStr">
         <is>
           <t>Orbital epoch</t>
         </is>
       </c>
-      <c r="BL1" s="1" t="inlineStr">
+      <c r="BM1" s="1" t="inlineStr">
         <is>
           <t>Orbital epoch_err</t>
         </is>
       </c>
-      <c r="BM1" s="1" t="inlineStr">
+      <c r="BN1" s="1" t="inlineStr">
         <is>
           <t>Ps</t>
         </is>
       </c>
-      <c r="BN1" s="1" t="inlineStr">
+      <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>e</t>
         </is>
       </c>
-      <c r="BO1" s="1" t="inlineStr">
+      <c r="BP1" s="1" t="inlineStr">
         <is>
           <t>e_err</t>
         </is>
       </c>
-      <c r="BP1" s="1" t="inlineStr">
+      <c r="BQ1" s="1" t="inlineStr">
         <is>
           <t>semi_eclipse</t>
         </is>
       </c>
-      <c r="BQ1" s="1" t="inlineStr">
+      <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>semi_eclipse_err</t>
         </is>
       </c>
-      <c r="BR1" s="1" t="inlineStr">
+      <c r="BS1" s="1" t="inlineStr">
         <is>
           <t>vsin(i)</t>
         </is>
       </c>
-      <c r="BS1" s="1" t="inlineStr">
+      <c r="BT1" s="1" t="inlineStr">
         <is>
           <t>vsin(i)_err</t>
         </is>
       </c>
-      <c r="BT1" s="1" t="inlineStr">
+      <c r="BU1" s="1" t="inlineStr">
         <is>
           <t>Mhrd</t>
         </is>
       </c>
-      <c r="BU1" s="1" t="inlineStr">
+      <c r="BV1" s="1" t="inlineStr">
         <is>
           <t>Mhrd_err</t>
         </is>
       </c>
-      <c r="BV1" s="1" t="inlineStr">
+      <c r="BW1" s="1" t="inlineStr">
         <is>
           <t>Lx</t>
         </is>
@@ -893,165 +898,168 @@
       <c r="Y2" t="n">
         <v>1000</v>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="Z2" t="n">
+        <v>27000</v>
+      </c>
+      <c r="AA2" t="inlineStr">
         <is>
           <t>12.4761106049604</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t>1.58367109395482</t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>1.28174948957142</t>
         </is>
       </c>
-      <c r="AC2" t="n">
+      <c r="AD2" t="n">
         <v>11.4</v>
       </c>
-      <c r="AD2" t="n">
+      <c r="AE2" t="n">
         <v>0.7</v>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
         <is>
           <t>14.36</t>
         </is>
       </c>
-      <c r="AF2" t="n">
+      <c r="AG2" t="n">
         <v>2.154</v>
       </c>
-      <c r="AG2" t="n">
+      <c r="AH2" t="n">
         <v>12.726</v>
       </c>
-      <c r="AH2" t="n">
+      <c r="AI2" t="n">
         <v>0.3229674906240564</v>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>12.3332840935839</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>0.293733098903704</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>6.36984218288446</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>0.181277751759849</t>
         </is>
       </c>
-      <c r="AM2" t="n">
+      <c r="AN2" t="n">
         <v>414.317</v>
       </c>
-      <c r="AN2" t="n">
+      <c r="AO2" t="n">
         <v>0.008999999999999999</v>
       </c>
-      <c r="AO2" t="n">
+      <c r="AP2" t="n">
         <v>28</v>
       </c>
-      <c r="AP2" t="n">
+      <c r="AQ2" t="n">
         <v>2</v>
       </c>
-      <c r="AQ2" t="n">
+      <c r="AR2" t="n">
         <v>0.066</v>
       </c>
-      <c r="AR2" t="n">
+      <c r="AS2" t="n">
         <v>0.005</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="AT2" t="n">
         <v>0.75</v>
       </c>
-      <c r="AT2" t="n">
+      <c r="AU2" t="n">
         <v>0.13</v>
       </c>
-      <c r="AU2" t="n">
+      <c r="AV2" t="n">
         <v>65</v>
       </c>
-      <c r="AV2" t="n">
+      <c r="AW2" t="n">
         <v>1</v>
       </c>
-      <c r="AW2" t="n">
+      <c r="AX2" t="n">
         <v>1.57</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="AY2" t="n">
         <v>0.16</v>
       </c>
-      <c r="AY2" t="n">
+      <c r="AZ2" t="n">
         <v>24</v>
       </c>
-      <c r="AZ2" t="n">
+      <c r="BA2" t="n">
         <v>1</v>
       </c>
-      <c r="BA2" t="n">
+      <c r="BB2" t="n">
         <v>0.63</v>
       </c>
-      <c r="BB2" t="n">
+      <c r="BC2" t="n">
         <v>0.01</v>
       </c>
-      <c r="BC2" t="n">
+      <c r="BD2" t="n">
         <v>20.2</v>
       </c>
-      <c r="BD2" t="n">
+      <c r="BE2" t="n">
         <v>0.4</v>
       </c>
-      <c r="BE2" t="n">
+      <c r="BF2" t="n">
         <v>50506.788423</v>
       </c>
-      <c r="BF2" t="n">
+      <c r="BG2" t="n">
         <v>7e-06</v>
       </c>
-      <c r="BG2" t="n">
+      <c r="BH2" t="n">
         <v>2.08704106</v>
       </c>
-      <c r="BH2" t="n">
+      <c r="BI2" t="n">
         <v>3e-08</v>
       </c>
-      <c r="BI2" t="n">
+      <c r="BJ2" t="n">
         <v>-1.8</v>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BK2" t="n">
         <v>0.001</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BL2" t="n">
         <v>50506.788423</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BM2" t="n">
         <v>7e-06</v>
       </c>
-      <c r="BM2" t="n">
+      <c r="BN2" t="n">
         <v>4.8</v>
       </c>
-      <c r="BN2" t="n">
+      <c r="BO2" t="n">
         <v>0.0016</v>
       </c>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="n">
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="n">
         <v>27.9</v>
       </c>
-      <c r="BQ2" t="n">
+      <c r="BR2" t="n">
         <v>0.3</v>
       </c>
-      <c r="BR2" t="n">
+      <c r="BS2" t="n">
         <v>204.8</v>
       </c>
-      <c r="BS2" t="n">
+      <c r="BT2" t="n">
         <v>0.8</v>
       </c>
-      <c r="BT2" t="n">
+      <c r="BU2" t="n">
         <v>29</v>
       </c>
-      <c r="BU2" t="n">
+      <c r="BV2" t="n">
         <v>2</v>
       </c>
-      <c r="BV2" t="n">
+      <c r="BW2" t="n">
         <v>5e+37</v>
       </c>
     </row>
@@ -1151,167 +1159,170 @@
       <c r="Y3" t="n">
         <v>1000</v>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z3" t="n">
+        <v>28000</v>
+      </c>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>29.8247550772236</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
+      <c r="AB3" t="inlineStr">
         <is>
           <t>3.59402714904720</t>
         </is>
       </c>
-      <c r="AB3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>3.87806883113850</t>
         </is>
       </c>
-      <c r="AC3" t="n">
+      <c r="AD3" t="n">
         <v>13</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AE3" t="n">
         <v>1</v>
       </c>
-      <c r="AE3" t="inlineStr">
+      <c r="AF3" t="inlineStr">
         <is>
           <t>22.599999999999994</t>
         </is>
       </c>
-      <c r="AF3" t="n">
+      <c r="AG3" t="n">
         <v>3.389999999999999</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AH3" t="n">
         <v>11.66</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="AI3" t="n">
         <v>0.8464632301523793</v>
       </c>
-      <c r="AI3" t="inlineStr">
+      <c r="AJ3" t="inlineStr">
         <is>
           <t>13.4738464692258</t>
         </is>
       </c>
-      <c r="AJ3" t="inlineStr">
+      <c r="AK3" t="inlineStr">
         <is>
           <t>0.697890522579867</t>
         </is>
       </c>
-      <c r="AK3" t="inlineStr">
+      <c r="AL3" t="inlineStr">
         <is>
           <t>7.96322282646401</t>
         </is>
       </c>
-      <c r="AL3" t="inlineStr">
+      <c r="AM3" t="inlineStr">
         <is>
           <t>0.457908402696324</t>
         </is>
       </c>
-      <c r="AM3" t="n">
+      <c r="AN3" t="n">
         <v>316</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="AO3" t="n">
         <v>10</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="AP3" t="n">
         <v>20</v>
       </c>
-      <c r="AP3" t="n">
+      <c r="AQ3" t="n">
         <v>3</v>
       </c>
-      <c r="AQ3" t="n">
+      <c r="AR3" t="n">
         <v>0.06</v>
       </c>
-      <c r="AR3" t="n">
+      <c r="AS3" t="n">
         <v>0.01</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="AT3" t="n">
         <v>0.91</v>
       </c>
-      <c r="AT3" t="n">
+      <c r="AU3" t="n">
         <v>0.2</v>
       </c>
-      <c r="AU3" t="n">
+      <c r="AV3" t="n">
         <v>67</v>
       </c>
-      <c r="AV3" t="n">
+      <c r="AW3" t="n">
         <v>1</v>
       </c>
-      <c r="AW3" t="n">
+      <c r="AX3" t="n">
         <v>1.02</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="AY3" t="n">
         <v>0.17</v>
       </c>
-      <c r="AY3" t="n">
+      <c r="AZ3" t="n">
         <v>16</v>
       </c>
-      <c r="AZ3" t="n">
+      <c r="BA3" t="n">
         <v>2</v>
       </c>
-      <c r="BA3" t="n">
+      <c r="BB3" t="n">
         <v>0.53</v>
       </c>
-      <c r="BB3" t="n">
+      <c r="BC3" t="n">
         <v>0.03</v>
       </c>
-      <c r="BC3" t="n">
+      <c r="BD3" t="n">
         <v>22</v>
       </c>
-      <c r="BD3" t="n">
+      <c r="BE3" t="n">
         <v>1</v>
       </c>
-      <c r="BE3" t="n">
+      <c r="BF3" t="n">
         <v>52855.061</v>
       </c>
-      <c r="BF3" t="n">
+      <c r="BG3" t="n">
         <v>0.013</v>
       </c>
-      <c r="BG3" t="n">
+      <c r="BH3" t="n">
         <v>3.728414</v>
       </c>
-      <c r="BH3" t="n">
+      <c r="BI3" t="n">
         <v>7.6e-06</v>
       </c>
-      <c r="BI3" t="n">
+      <c r="BJ3" t="n">
         <v>-0.7</v>
       </c>
-      <c r="BJ3" t="n">
+      <c r="BK3" t="n">
         <v>0.8</v>
       </c>
-      <c r="BK3" t="n">
+      <c r="BL3" t="n">
         <v>52851.33</v>
       </c>
-      <c r="BL3" t="n">
+      <c r="BM3" t="n">
         <v>0.01</v>
       </c>
-      <c r="BM3" t="n">
+      <c r="BN3" t="n">
         <v>526.8</v>
       </c>
-      <c r="BN3" t="n">
+      <c r="BO3" t="n">
         <v>0.18</v>
       </c>
-      <c r="BO3" t="n">
+      <c r="BP3" t="n">
         <v>0.01</v>
       </c>
-      <c r="BP3" t="n">
+      <c r="BQ3" t="n">
         <v>21</v>
       </c>
-      <c r="BQ3" t="n">
+      <c r="BR3" t="n">
         <v>1</v>
       </c>
-      <c r="BR3" t="n">
+      <c r="BS3" t="n">
         <v>224.9</v>
       </c>
-      <c r="BS3" t="n">
+      <c r="BT3" t="n">
         <v>0.7</v>
       </c>
-      <c r="BT3" t="n">
-        <v>35</v>
-      </c>
       <c r="BU3" t="n">
+        <v>29</v>
+      </c>
+      <c r="BV3" t="n">
         <v>2</v>
       </c>
-      <c r="BV3" t="n">
+      <c r="BW3" t="n">
         <v>2e+36</v>
       </c>
     </row>
@@ -1413,157 +1424,160 @@
       <c r="Y4" t="n">
         <v>1000</v>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="Z4" t="n">
+        <v>30000</v>
+      </c>
+      <c r="AA4" t="inlineStr">
         <is>
           <t>16.9632541964421</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>1.51028021716036</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>1.36297188049476</t>
         </is>
       </c>
-      <c r="AC4" t="n">
+      <c r="AD4" t="n">
         <v>22</v>
       </c>
-      <c r="AD4" t="n">
+      <c r="AE4" t="n">
         <v>2</v>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
         <is>
           <t>20.22</t>
         </is>
       </c>
-      <c r="AF4" t="n">
+      <c r="AG4" t="n">
         <v>3.033</v>
       </c>
-      <c r="AG4" t="n">
+      <c r="AH4" t="n">
         <v>24.29</v>
       </c>
-      <c r="AH4" t="n">
+      <c r="AI4" t="n">
         <v>0.7250765476830705</v>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>22.4221610513527</t>
         </is>
       </c>
-      <c r="AJ4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>0.725547330706974</t>
         </is>
       </c>
-      <c r="AK4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>11.0576539439844</t>
         </is>
       </c>
-      <c r="AL4" t="inlineStr">
+      <c r="AM4" t="inlineStr">
         <is>
           <t>0.534214506648961</t>
         </is>
       </c>
-      <c r="AM4" t="n">
+      <c r="AN4" t="n">
         <v>435</v>
       </c>
-      <c r="AN4" t="n">
+      <c r="AO4" t="n">
         <v>10</v>
       </c>
-      <c r="AO4" t="n">
+      <c r="AP4" t="n">
         <v>19</v>
       </c>
-      <c r="AP4" t="n">
+      <c r="AQ4" t="n">
         <v>1</v>
       </c>
-      <c r="AQ4" t="n">
+      <c r="AR4" t="n">
         <v>0.043</v>
       </c>
-      <c r="AR4" t="n">
+      <c r="AS4" t="n">
         <v>0.002</v>
       </c>
-      <c r="AS4" t="n">
+      <c r="AT4" t="n">
         <v>0.47</v>
       </c>
-      <c r="AT4" t="n">
+      <c r="AU4" t="n">
         <v>0.04</v>
       </c>
-      <c r="AU4" t="n">
+      <c r="AV4" t="n">
         <v>62</v>
       </c>
-      <c r="AV4" t="n">
+      <c r="AW4" t="n">
         <v>1</v>
       </c>
-      <c r="AW4" t="n">
+      <c r="AX4" t="n">
         <v>1.96</v>
       </c>
-      <c r="AX4" t="n">
+      <c r="AY4" t="n">
         <v>0.19</v>
       </c>
-      <c r="AY4" t="n">
+      <c r="AZ4" t="n">
         <v>46</v>
       </c>
-      <c r="AZ4" t="n">
+      <c r="BA4" t="n">
         <v>5</v>
       </c>
-      <c r="BA4" t="n">
+      <c r="BB4" t="n">
         <v>0.694</v>
       </c>
-      <c r="BB4" t="n">
+      <c r="BC4" t="n">
         <v>0.006</v>
       </c>
-      <c r="BC4" t="n">
+      <c r="BD4" t="n">
         <v>35</v>
       </c>
-      <c r="BD4" t="n">
+      <c r="BE4" t="n">
         <v>1</v>
       </c>
-      <c r="BE4" t="n">
+      <c r="BF4" t="n">
         <v>53785.85</v>
       </c>
-      <c r="BF4" t="n">
+      <c r="BG4" t="n">
         <v>0.007</v>
       </c>
-      <c r="BG4" t="n">
+      <c r="BH4" t="n">
         <v>3.411581</v>
       </c>
-      <c r="BH4" t="n">
+      <c r="BI4" t="n">
         <v>7e-06</v>
       </c>
-      <c r="BI4" t="n">
+      <c r="BJ4" t="n">
         <v>-1.6</v>
       </c>
-      <c r="BJ4" t="n">
+      <c r="BK4" t="n">
         <v>0.1</v>
       </c>
-      <c r="BK4" t="n">
+      <c r="BL4" t="n">
         <v>48900.373</v>
       </c>
-      <c r="BL4" t="n">
+      <c r="BM4" t="n">
         <v>0.015</v>
       </c>
-      <c r="BM4" t="inlineStr"/>
       <c r="BN4" t="inlineStr"/>
       <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="n">
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="n">
         <v>32</v>
       </c>
-      <c r="BQ4" t="n">
+      <c r="BR4" t="n">
         <v>1</v>
       </c>
-      <c r="BR4" t="inlineStr"/>
       <c r="BS4" t="inlineStr"/>
-      <c r="BT4" t="n">
-        <v>44</v>
-      </c>
+      <c r="BT4" t="inlineStr"/>
       <c r="BU4" t="n">
+        <v>41</v>
+      </c>
+      <c r="BV4" t="n">
         <v>2</v>
       </c>
-      <c r="BV4" t="n">
+      <c r="BW4" t="n">
         <v>9.800000000000001e+35</v>
       </c>
     </row>
@@ -1665,167 +1679,170 @@
       <c r="Y5" t="n">
         <v>1000</v>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="Z5" t="n">
+        <v>31000</v>
+      </c>
+      <c r="AA5" t="inlineStr">
         <is>
           <t>9.78778771242834</t>
         </is>
       </c>
-      <c r="AA5" t="inlineStr">
+      <c r="AB5" t="inlineStr">
         <is>
           <t>1.11222907861592</t>
         </is>
       </c>
-      <c r="AB5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>1.11222907861592</t>
         </is>
       </c>
-      <c r="AC5" t="n">
+      <c r="AD5" t="n">
         <v>7.4</v>
       </c>
-      <c r="AD5" t="n">
+      <c r="AE5" t="n">
         <v>0.4</v>
       </c>
-      <c r="AE5" t="inlineStr">
+      <c r="AF5" t="inlineStr">
         <is>
           <t>13.74</t>
         </is>
       </c>
-      <c r="AF5" t="n">
+      <c r="AG5" t="n">
         <v>2.061</v>
       </c>
-      <c r="AG5" t="n">
+      <c r="AH5" t="n">
         <v>8.377999999999998</v>
       </c>
-      <c r="AH5" t="n">
+      <c r="AI5" t="n">
         <v>0.1846293584455083</v>
       </c>
-      <c r="AI5" t="inlineStr">
+      <c r="AJ5" t="inlineStr">
         <is>
           <t>8.36188984223463</t>
         </is>
       </c>
-      <c r="AJ5" t="inlineStr">
+      <c r="AK5" t="inlineStr">
         <is>
           <t>0.153362041572946</t>
         </is>
       </c>
-      <c r="AK5" t="inlineStr">
+      <c r="AL5" t="inlineStr">
         <is>
           <t>4.29964416954258</t>
         </is>
       </c>
-      <c r="AL5" t="inlineStr">
+      <c r="AM5" t="inlineStr">
         <is>
           <t>0.113170143887694</t>
         </is>
       </c>
-      <c r="AM5" t="n">
+      <c r="AN5" t="n">
         <v>407.8</v>
       </c>
-      <c r="AN5" t="n">
+      <c r="AO5" t="n">
         <v>0.3</v>
       </c>
-      <c r="AO5" t="n">
+      <c r="AP5" t="n">
         <v>35</v>
       </c>
-      <c r="AP5" t="n">
+      <c r="AQ5" t="n">
         <v>2</v>
       </c>
-      <c r="AQ5" t="n">
+      <c r="AR5" t="n">
         <v>0.08599999999999999</v>
       </c>
-      <c r="AR5" t="n">
+      <c r="AS5" t="n">
         <v>0.004</v>
       </c>
-      <c r="AS5" t="n">
+      <c r="AT5" t="n">
         <v>0.97</v>
       </c>
-      <c r="AT5" t="n">
+      <c r="AU5" t="n">
         <v>0.13</v>
       </c>
-      <c r="AU5" t="n">
+      <c r="AV5" t="n">
         <v>59.3</v>
       </c>
-      <c r="AV5" t="n">
+      <c r="AW5" t="n">
         <v>0.9</v>
       </c>
-      <c r="AW5" t="n">
+      <c r="AX5" t="n">
         <v>1.57</v>
       </c>
-      <c r="AX5" t="n">
+      <c r="AY5" t="n">
         <v>0.11</v>
       </c>
-      <c r="AY5" t="n">
+      <c r="AZ5" t="n">
         <v>18</v>
       </c>
-      <c r="AZ5" t="n">
+      <c r="BA5" t="n">
         <v>1</v>
       </c>
-      <c r="BA5" t="n">
+      <c r="BB5" t="n">
         <v>0.59</v>
       </c>
-      <c r="BB5" t="n">
+      <c r="BC5" t="n">
         <v>0.01</v>
       </c>
-      <c r="BC5" t="n">
+      <c r="BD5" t="n">
         <v>14.2</v>
       </c>
-      <c r="BD5" t="n">
+      <c r="BE5" t="n">
         <v>0.2</v>
       </c>
-      <c r="BE5" t="n">
+      <c r="BF5" t="n">
         <v>53013.591</v>
       </c>
-      <c r="BF5" t="n">
+      <c r="BG5" t="n">
         <v>0.0008</v>
       </c>
-      <c r="BG5" t="n">
+      <c r="BH5" t="n">
         <v>1.408379</v>
       </c>
-      <c r="BH5" t="n">
+      <c r="BI5" t="n">
         <v>7e-07</v>
       </c>
-      <c r="BI5" t="n">
+      <c r="BJ5" t="n">
         <v>-1</v>
       </c>
-      <c r="BJ5" t="n">
+      <c r="BK5" t="n">
         <v>0.05</v>
       </c>
-      <c r="BK5" t="n">
+      <c r="BL5" t="n">
         <v>51110.86579</v>
       </c>
-      <c r="BL5" t="n">
+      <c r="BM5" t="n">
         <v>0.0001</v>
       </c>
-      <c r="BM5" t="n">
+      <c r="BN5" t="n">
         <v>13.5</v>
       </c>
-      <c r="BN5" t="n">
+      <c r="BO5" t="n">
         <v>0.006</v>
       </c>
-      <c r="BO5" t="n">
+      <c r="BP5" t="n">
         <v>0.002</v>
       </c>
-      <c r="BP5" t="n">
+      <c r="BQ5" t="n">
         <v>15.8</v>
       </c>
-      <c r="BQ5" t="n">
+      <c r="BR5" t="n">
         <v>0.8</v>
       </c>
-      <c r="BR5" t="n">
+      <c r="BS5" t="n">
         <v>257.9</v>
       </c>
-      <c r="BS5" t="n">
+      <c r="BT5" t="n">
         <v>0.7</v>
       </c>
-      <c r="BT5" t="n">
+      <c r="BU5" t="n">
         <v>22</v>
       </c>
-      <c r="BU5" t="n">
+      <c r="BV5" t="n">
         <v>1</v>
       </c>
-      <c r="BV5" t="n">
+      <c r="BW5" t="n">
         <v>2.2e+38</v>
       </c>
     </row>
@@ -1925,167 +1942,170 @@
       <c r="Y6" t="n">
         <v>1000</v>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="Z6" t="n">
+        <v>23000</v>
+      </c>
+      <c r="AA6" t="inlineStr">
         <is>
           <t>24.4179192218864</t>
         </is>
       </c>
-      <c r="AA6" t="inlineStr">
+      <c r="AB6" t="inlineStr">
         <is>
           <t>2.79595751310347</t>
         </is>
       </c>
-      <c r="AB6" t="inlineStr">
+      <c r="AC6" t="inlineStr">
         <is>
           <t>2.79595751310347</t>
         </is>
       </c>
-      <c r="AC6" t="n">
+      <c r="AD6" t="n">
         <v>15</v>
       </c>
-      <c r="AD6" t="n">
+      <c r="AE6" t="n">
         <v>1</v>
       </c>
-      <c r="AE6" t="inlineStr">
+      <c r="AF6" t="inlineStr">
         <is>
           <t>22.459999999999997</t>
         </is>
       </c>
-      <c r="AF6" t="n">
+      <c r="AG6" t="n">
         <v>3.368999999999999</v>
       </c>
-      <c r="AG6" t="n">
+      <c r="AH6" t="n">
         <v>17.019</v>
       </c>
-      <c r="AH6" t="n">
+      <c r="AI6" t="n">
         <v>0.7026329055773007</v>
       </c>
-      <c r="AI6" t="inlineStr">
+      <c r="AJ6" t="inlineStr">
         <is>
           <t>16.9786936673335</t>
         </is>
       </c>
-      <c r="AJ6" t="inlineStr">
+      <c r="AK6" t="inlineStr">
         <is>
           <t>0.524823344586292</t>
         </is>
       </c>
-      <c r="AK6" t="inlineStr">
+      <c r="AL6" t="inlineStr">
         <is>
           <t>10.1601686470543</t>
         </is>
       </c>
-      <c r="AL6" t="inlineStr">
+      <c r="AM6" t="inlineStr">
         <is>
           <t>0.404455984912469</t>
         </is>
       </c>
-      <c r="AM6" t="n">
+      <c r="AN6" t="n">
         <v>299.631</v>
       </c>
-      <c r="AN6" t="n">
+      <c r="AO6" t="n">
         <v>0.005</v>
       </c>
-      <c r="AO6" t="n">
+      <c r="AP6" t="n">
         <v>20</v>
       </c>
-      <c r="AP6" t="n">
+      <c r="AQ6" t="n">
         <v>1</v>
       </c>
-      <c r="AQ6" t="n">
+      <c r="AR6" t="n">
         <v>0.067</v>
       </c>
-      <c r="AR6" t="n">
+      <c r="AS6" t="n">
         <v>0.004</v>
       </c>
-      <c r="AS6" t="n">
+      <c r="AT6" t="n">
         <v>0.91</v>
       </c>
-      <c r="AT6" t="n">
+      <c r="AU6" t="n">
         <v>0.2</v>
       </c>
-      <c r="AU6" t="n">
+      <c r="AV6" t="n">
         <v>62</v>
       </c>
-      <c r="AV6" t="n">
+      <c r="AW6" t="n">
         <v>2</v>
       </c>
-      <c r="AW6" t="n">
+      <c r="AX6" t="n">
         <v>1.21</v>
       </c>
-      <c r="AX6" t="n">
+      <c r="AY6" t="n">
         <v>0.12</v>
       </c>
-      <c r="AY6" t="n">
+      <c r="AZ6" t="n">
         <v>18</v>
       </c>
-      <c r="AZ6" t="n">
+      <c r="BA6" t="n">
         <v>2</v>
       </c>
-      <c r="BA6" t="n">
+      <c r="BB6" t="n">
         <v>0.61</v>
       </c>
-      <c r="BB6" t="n">
+      <c r="BC6" t="n">
         <v>0.02</v>
       </c>
-      <c r="BC6" t="n">
+      <c r="BD6" t="n">
         <v>27.9</v>
       </c>
-      <c r="BD6" t="n">
+      <c r="BE6" t="n">
         <v>0.7</v>
       </c>
-      <c r="BE6" t="n">
+      <c r="BF6" t="n">
         <v>52846.68881</v>
       </c>
-      <c r="BF6" t="n">
+      <c r="BG6" t="n">
         <v>2.4e-05</v>
       </c>
-      <c r="BG6" t="n">
+      <c r="BH6" t="n">
         <v>3.89192316</v>
       </c>
-      <c r="BH6" t="n">
+      <c r="BI6" t="n">
         <v>6.6e-08</v>
       </c>
-      <c r="BI6" t="n">
+      <c r="BJ6" t="n">
         <v>-3.541</v>
       </c>
-      <c r="BJ6" t="n">
+      <c r="BK6" t="n">
         <v>0.002</v>
       </c>
-      <c r="BK6" t="n">
+      <c r="BL6" t="n">
         <v>50324.691861</v>
       </c>
-      <c r="BL6" t="n">
+      <c r="BM6" t="n">
         <v>8e-06</v>
       </c>
-      <c r="BM6" t="n">
+      <c r="BN6" t="n">
         <v>0.71</v>
       </c>
-      <c r="BN6" t="n">
+      <c r="BO6" t="n">
         <v>0.0008899999999999999</v>
       </c>
-      <c r="BO6" t="n">
+      <c r="BP6" t="n">
         <v>6e-05</v>
       </c>
-      <c r="BP6" t="n">
+      <c r="BQ6" t="n">
         <v>23</v>
       </c>
-      <c r="BQ6" t="n">
+      <c r="BR6" t="n">
         <v>2</v>
       </c>
-      <c r="BR6" t="n">
+      <c r="BS6" t="n">
         <v>178</v>
       </c>
-      <c r="BS6" t="n">
+      <c r="BT6" t="n">
         <v>0.8</v>
       </c>
-      <c r="BT6" t="n">
-        <v>29</v>
-      </c>
       <c r="BU6" t="n">
+        <v>23</v>
+      </c>
+      <c r="BV6" t="n">
         <v>2</v>
       </c>
-      <c r="BV6" t="n">
+      <c r="BW6" t="n">
         <v>2.6e+38</v>
       </c>
     </row>
@@ -2185,167 +2205,170 @@
       <c r="Y7" t="n">
         <v>1000</v>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="Z7" t="n">
+        <v>20000</v>
+      </c>
+      <c r="AA7" t="inlineStr">
         <is>
           <t>40.7448210535303</t>
         </is>
       </c>
-      <c r="AA7" t="inlineStr">
+      <c r="AB7" t="inlineStr">
         <is>
           <t>4.28223176063543</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
+      <c r="AC7" t="inlineStr">
         <is>
           <t>4.33270047297629</t>
         </is>
       </c>
-      <c r="AC7" t="n">
+      <c r="AD7" t="n">
         <v>29</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AE7" t="n">
         <v>1</v>
       </c>
-      <c r="AE7" t="inlineStr">
+      <c r="AF7" t="inlineStr">
         <is>
           <t>22.809999999999995</t>
         </is>
       </c>
-      <c r="AF7" t="n">
+      <c r="AG7" t="n">
         <v>3.421499999999999</v>
       </c>
-      <c r="AG7" t="n">
+      <c r="AH7" t="n">
         <v>35.462</v>
       </c>
-      <c r="AH7" t="n">
+      <c r="AI7" t="n">
         <v>0.5489535590557729</v>
       </c>
-      <c r="AI7" t="inlineStr">
+      <c r="AJ7" t="inlineStr">
         <is>
           <t>35.4052971460730</t>
         </is>
       </c>
-      <c r="AJ7" t="inlineStr">
+      <c r="AK7" t="inlineStr">
         <is>
           <t>0.567412643709415</t>
         </is>
       </c>
-      <c r="AK7" t="inlineStr">
+      <c r="AL7" t="inlineStr">
         <is>
           <t>23.2133018271434</t>
         </is>
       </c>
-      <c r="AL7" t="inlineStr">
+      <c r="AM7" t="inlineStr">
         <is>
           <t>0.381892414835567</t>
         </is>
       </c>
-      <c r="AM7" t="n">
+      <c r="AN7" t="n">
         <v>278.1</v>
       </c>
-      <c r="AN7" t="n">
+      <c r="AO7" t="n">
         <v>0.3</v>
       </c>
-      <c r="AO7" t="n">
+      <c r="AP7" t="n">
         <v>23</v>
       </c>
-      <c r="AP7" t="n">
+      <c r="AQ7" t="n">
         <v>2</v>
       </c>
-      <c r="AQ7" t="n">
+      <c r="AR7" t="n">
         <v>0.081</v>
       </c>
-      <c r="AR7" t="n">
+      <c r="AS7" t="n">
         <v>0.005</v>
       </c>
-      <c r="AS7" t="n">
+      <c r="AT7" t="n">
         <v>0.67</v>
       </c>
-      <c r="AT7" t="n">
+      <c r="AU7" t="n">
         <v>0.04</v>
       </c>
-      <c r="AU7" t="n">
+      <c r="AV7" t="n">
         <v>72.8</v>
       </c>
-      <c r="AV7" t="n">
+      <c r="AW7" t="n">
         <v>0.4</v>
       </c>
-      <c r="AW7" t="n">
+      <c r="AX7" t="n">
         <v>2.12</v>
       </c>
-      <c r="AX7" t="n">
+      <c r="AY7" t="n">
         <v>0.16</v>
       </c>
-      <c r="AY7" t="n">
+      <c r="AZ7" t="n">
         <v>26</v>
       </c>
-      <c r="AZ7" t="n">
+      <c r="BA7" t="n">
         <v>1</v>
       </c>
-      <c r="BA7" t="n">
+      <c r="BB7" t="n">
         <v>0.595</v>
       </c>
-      <c r="BB7" t="n">
+      <c r="BC7" t="n">
         <v>0.006</v>
       </c>
-      <c r="BC7" t="n">
+      <c r="BD7" t="n">
         <v>59.6</v>
       </c>
-      <c r="BD7" t="n">
+      <c r="BE7" t="n">
         <v>0.7</v>
       </c>
-      <c r="BE7" t="n">
+      <c r="BF7" t="n">
         <v>42611.349</v>
       </c>
-      <c r="BF7" t="n">
+      <c r="BG7" t="n">
         <v>0.013</v>
       </c>
-      <c r="BG7" t="n">
+      <c r="BH7" t="n">
         <v>8.964427000000001</v>
       </c>
-      <c r="BH7" t="n">
+      <c r="BI7" t="n">
         <v>1.2e-05</v>
       </c>
-      <c r="BI7" t="n">
+      <c r="BJ7" t="n">
         <v>-0.1</v>
       </c>
-      <c r="BJ7" t="n">
+      <c r="BK7" t="n">
         <v>0.3</v>
       </c>
-      <c r="BK7" t="n">
+      <c r="BL7" t="n">
         <v>48895.2186</v>
       </c>
-      <c r="BL7" t="n">
+      <c r="BM7" t="n">
         <v>0.0012</v>
       </c>
-      <c r="BM7" t="n">
+      <c r="BN7" t="n">
         <v>283.2</v>
       </c>
-      <c r="BN7" t="n">
+      <c r="BO7" t="n">
         <v>0.0898</v>
       </c>
-      <c r="BO7" t="n">
+      <c r="BP7" t="n">
         <v>0.0012</v>
       </c>
-      <c r="BP7" t="n">
+      <c r="BQ7" t="n">
         <v>30.5</v>
       </c>
-      <c r="BQ7" t="n">
+      <c r="BR7" t="n">
         <v>0.1</v>
       </c>
-      <c r="BR7" t="n">
+      <c r="BS7" t="n">
         <v>130.3</v>
       </c>
-      <c r="BS7" t="n">
+      <c r="BT7" t="n">
         <v>0.2</v>
       </c>
-      <c r="BT7" t="n">
-        <v>42</v>
-      </c>
       <c r="BU7" t="n">
+        <v>32</v>
+      </c>
+      <c r="BV7" t="n">
         <v>2</v>
       </c>
-      <c r="BV7" t="n">
+      <c r="BW7" t="n">
         <v>4.6e+36</v>
       </c>
     </row>

</xml_diff>